<commit_message>
update of prematch statistics
</commit_message>
<xml_diff>
--- a/datasets/xlsx/CSPreMatchStatistics.xlsx
+++ b/datasets/xlsx/CSPreMatchStatistics.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexPost\Repos\HardWareWebsite\datasets\xlsx\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexPost\repos\HardWareWebsite\datasets\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36374337-28A4-44A8-9467-76AFC1A84332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B12050F-519B-4520-A506-AF3D151ADA60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="38">
   <si>
     <t>ID</t>
   </si>
@@ -149,6 +149,9 @@
   <si>
     <t>AnubisDiff</t>
   </si>
+  <si>
+    <t>CacheDiff</t>
+  </si>
 </sst>
 </file>
 
@@ -209,10 +212,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -478,28 +477,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U266"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:V267"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="14.85546875" customWidth="1"/>
-    <col min="3" max="3" width="13.28515625" customWidth="1"/>
-    <col min="4" max="5" width="13.5703125" customWidth="1"/>
-    <col min="6" max="6" width="12.28515625" customWidth="1"/>
+    <col min="2" max="2" width="14.88671875" customWidth="1"/>
+    <col min="3" max="3" width="13.33203125" customWidth="1"/>
+    <col min="4" max="5" width="13.5546875" customWidth="1"/>
+    <col min="6" max="6" width="12.33203125" customWidth="1"/>
     <col min="7" max="7" width="12" customWidth="1"/>
-    <col min="8" max="8" width="12.5703125" customWidth="1"/>
-    <col min="9" max="9" width="11.28515625" customWidth="1"/>
-    <col min="10" max="10" width="10.5703125" customWidth="1"/>
+    <col min="8" max="8" width="12.5546875" customWidth="1"/>
+    <col min="9" max="9" width="11.33203125" customWidth="1"/>
+    <col min="10" max="10" width="10.5546875" customWidth="1"/>
     <col min="11" max="11" width="11" customWidth="1"/>
-    <col min="12" max="13" width="10.42578125" customWidth="1"/>
-    <col min="14" max="14" width="11.5703125" customWidth="1"/>
-    <col min="15" max="15" width="10.42578125" customWidth="1"/>
-    <col min="17" max="17" width="9.5703125" customWidth="1"/>
-    <col min="19" max="19" width="11.7109375" customWidth="1"/>
-    <col min="20" max="20" width="12.85546875" customWidth="1"/>
-    <col min="21" max="21" width="11.42578125" customWidth="1"/>
+    <col min="12" max="13" width="10.44140625" customWidth="1"/>
+    <col min="14" max="14" width="11.5546875" customWidth="1"/>
+    <col min="15" max="15" width="10.44140625" customWidth="1"/>
+    <col min="17" max="17" width="9.5546875" customWidth="1"/>
+    <col min="19" max="19" width="11.6640625" customWidth="1"/>
+    <col min="20" max="20" width="12.88671875" customWidth="1"/>
+    <col min="21" max="21" width="11.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -563,8 +562,11 @@
       <c r="U1" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>744</v>
       </c>
@@ -608,7 +610,7 @@
         <v>-6</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>745</v>
       </c>
@@ -649,7 +651,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>750</v>
       </c>
@@ -699,7 +701,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>752</v>
       </c>
@@ -755,7 +757,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>753</v>
       </c>
@@ -814,7 +816,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>754</v>
       </c>
@@ -870,7 +872,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>755</v>
       </c>
@@ -926,7 +928,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>756</v>
       </c>
@@ -982,7 +984,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>757</v>
       </c>
@@ -1026,7 +1028,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>758</v>
       </c>
@@ -1067,7 +1069,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>759</v>
       </c>
@@ -1120,7 +1122,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>760</v>
       </c>
@@ -1176,7 +1178,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>761</v>
       </c>
@@ -1238,7 +1240,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>762</v>
       </c>
@@ -1291,7 +1293,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>763</v>
       </c>
@@ -1347,7 +1349,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>764</v>
       </c>
@@ -1406,7 +1408,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>765</v>
       </c>
@@ -1456,7 +1458,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>766</v>
       </c>
@@ -1500,7 +1502,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>767</v>
       </c>
@@ -1559,7 +1561,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>768</v>
       </c>
@@ -1615,7 +1617,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>769</v>
       </c>
@@ -1677,7 +1679,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>770</v>
       </c>
@@ -1736,7 +1738,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>771</v>
       </c>
@@ -1789,7 +1791,7 @@
         <v>-6</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>772</v>
       </c>
@@ -1836,7 +1838,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>773</v>
       </c>
@@ -1892,7 +1894,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>775</v>
       </c>
@@ -1951,7 +1953,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>776</v>
       </c>
@@ -2007,7 +2009,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>777</v>
       </c>
@@ -2069,7 +2071,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>780</v>
       </c>
@@ -2131,7 +2133,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>781</v>
       </c>
@@ -2190,7 +2192,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>782</v>
       </c>
@@ -2249,7 +2251,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>783</v>
       </c>
@@ -2308,7 +2310,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="34" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>784</v>
       </c>
@@ -2367,7 +2369,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="35" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>785</v>
       </c>
@@ -2426,7 +2428,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="36" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>786</v>
       </c>
@@ -2488,7 +2490,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="37" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>787</v>
       </c>
@@ -2544,7 +2546,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="38" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>788</v>
       </c>
@@ -2591,7 +2593,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="39" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>789</v>
       </c>
@@ -2647,7 +2649,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="40" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>790</v>
       </c>
@@ -2703,7 +2705,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="41" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>791</v>
       </c>
@@ -2759,7 +2761,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="42" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>792</v>
       </c>
@@ -2821,7 +2823,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="43" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>793</v>
       </c>
@@ -2883,7 +2885,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="44" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>794</v>
       </c>
@@ -2945,7 +2947,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="45" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>795</v>
       </c>
@@ -3004,7 +3006,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>796</v>
       </c>
@@ -3066,7 +3068,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="47" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>797</v>
       </c>
@@ -3122,7 +3124,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="48" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>798</v>
       </c>
@@ -3178,7 +3180,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="49" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>799</v>
       </c>
@@ -3231,7 +3233,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>800</v>
       </c>
@@ -3293,7 +3295,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="51" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>801</v>
       </c>
@@ -3352,7 +3354,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>802</v>
       </c>
@@ -3405,7 +3407,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="53" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>803</v>
       </c>
@@ -3458,7 +3460,7 @@
         <v>-13</v>
       </c>
     </row>
-    <row r="54" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>804</v>
       </c>
@@ -3520,7 +3522,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="55" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>805</v>
       </c>
@@ -3576,7 +3578,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="56" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>807</v>
       </c>
@@ -3629,7 +3631,7 @@
         <v>-8</v>
       </c>
     </row>
-    <row r="57" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>808</v>
       </c>
@@ -3685,7 +3687,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="58" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>809</v>
       </c>
@@ -3747,7 +3749,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="59" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>810</v>
       </c>
@@ -3806,7 +3808,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="60" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>811</v>
       </c>
@@ -3868,7 +3870,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="61" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>812</v>
       </c>
@@ -3927,7 +3929,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>813</v>
       </c>
@@ -3986,7 +3988,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="63" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>814</v>
       </c>
@@ -4042,7 +4044,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="64" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>815</v>
       </c>
@@ -4098,7 +4100,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="65" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>818</v>
       </c>
@@ -4145,7 +4147,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>819</v>
       </c>
@@ -4198,7 +4200,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="67" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>820</v>
       </c>
@@ -4257,7 +4259,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="68" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>821</v>
       </c>
@@ -4316,7 +4318,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="69" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>822</v>
       </c>
@@ -4372,7 +4374,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="70" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>823</v>
       </c>
@@ -4422,7 +4424,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="71" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>824</v>
       </c>
@@ -4481,7 +4483,7 @@
         <v>-6</v>
       </c>
     </row>
-    <row r="72" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>826</v>
       </c>
@@ -4540,7 +4542,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="73" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>827</v>
       </c>
@@ -4602,7 +4604,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>828</v>
       </c>
@@ -4658,7 +4660,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="75" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>830</v>
       </c>
@@ -4720,7 +4722,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>831</v>
       </c>
@@ -4776,7 +4778,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="77" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>832</v>
       </c>
@@ -4829,7 +4831,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="78" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>833</v>
       </c>
@@ -4891,7 +4893,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="79" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>834</v>
       </c>
@@ -4947,7 +4949,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="80" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>835</v>
       </c>
@@ -5009,7 +5011,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="81" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>836</v>
       </c>
@@ -5071,7 +5073,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="82" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>837</v>
       </c>
@@ -5133,7 +5135,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="83" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A83">
         <v>838</v>
       </c>
@@ -5195,7 +5197,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="84" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A84">
         <v>839</v>
       </c>
@@ -5254,7 +5256,7 @@
         <v>-8</v>
       </c>
     </row>
-    <row r="85" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>840</v>
       </c>
@@ -5316,7 +5318,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="86" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>841</v>
       </c>
@@ -5372,7 +5374,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="87" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>842</v>
       </c>
@@ -5431,7 +5433,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="88" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>843</v>
       </c>
@@ -5493,7 +5495,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="89" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A89">
         <v>844</v>
       </c>
@@ -5549,7 +5551,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A90">
         <v>845</v>
       </c>
@@ -5611,7 +5613,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="91" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A91">
         <v>846</v>
       </c>
@@ -5670,7 +5672,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="92" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A92">
         <v>848</v>
       </c>
@@ -5732,7 +5734,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="93" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A93">
         <v>850</v>
       </c>
@@ -5794,7 +5796,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="94" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A94">
         <v>851</v>
       </c>
@@ -5853,7 +5855,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="95" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A95">
         <v>853</v>
       </c>
@@ -5915,7 +5917,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="96" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A96">
         <v>854</v>
       </c>
@@ -5974,7 +5976,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="97" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A97">
         <v>855</v>
       </c>
@@ -6030,7 +6032,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="98" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A98">
         <v>856</v>
       </c>
@@ -6092,7 +6094,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="99" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A99">
         <v>857</v>
       </c>
@@ -6148,7 +6150,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A100">
         <v>859</v>
       </c>
@@ -6210,7 +6212,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="101" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A101">
         <v>860</v>
       </c>
@@ -6272,7 +6274,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="102" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A102">
         <v>861</v>
       </c>
@@ -6331,7 +6333,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="103" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A103">
         <v>862</v>
       </c>
@@ -6390,7 +6392,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="104" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A104">
         <v>863</v>
       </c>
@@ -6452,7 +6454,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="105" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A105">
         <v>864</v>
       </c>
@@ -6514,7 +6516,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="106" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A106">
         <v>865</v>
       </c>
@@ -6573,7 +6575,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="107" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A107">
         <v>866</v>
       </c>
@@ -6632,7 +6634,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="108" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A108">
         <v>867</v>
       </c>
@@ -6691,7 +6693,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="109" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A109">
         <v>868</v>
       </c>
@@ -6750,7 +6752,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="110" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A110">
         <v>869</v>
       </c>
@@ -6812,7 +6814,7 @@
         <v>-9</v>
       </c>
     </row>
-    <row r="111" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A111">
         <v>870</v>
       </c>
@@ -6874,7 +6876,7 @@
         <v>-9</v>
       </c>
     </row>
-    <row r="112" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A112">
         <v>871</v>
       </c>
@@ -6933,7 +6935,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="113" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A113">
         <v>872</v>
       </c>
@@ -6995,7 +6997,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="114" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A114">
         <v>873</v>
       </c>
@@ -7054,7 +7056,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="115" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A115">
         <v>874</v>
       </c>
@@ -7113,7 +7115,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A116">
         <v>875</v>
       </c>
@@ -7172,7 +7174,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="117" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A117">
         <v>876</v>
       </c>
@@ -7234,7 +7236,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="118" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A118">
         <v>877</v>
       </c>
@@ -7296,7 +7298,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="119" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A119">
         <v>878</v>
       </c>
@@ -7355,7 +7357,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="120" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A120">
         <v>880</v>
       </c>
@@ -7417,7 +7419,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A121">
         <v>881</v>
       </c>
@@ -7476,7 +7478,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="122" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A122">
         <v>882</v>
       </c>
@@ -7535,7 +7537,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="123" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A123">
         <v>883</v>
       </c>
@@ -7597,7 +7599,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="124" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A124">
         <v>884</v>
       </c>
@@ -7644,7 +7646,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="125" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A125">
         <v>885</v>
       </c>
@@ -7703,7 +7705,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="126" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A126">
         <v>886</v>
       </c>
@@ -7762,7 +7764,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="127" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A127">
         <v>887</v>
       </c>
@@ -7818,7 +7820,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A128">
         <v>888</v>
       </c>
@@ -7877,7 +7879,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="129" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A129">
         <v>889</v>
       </c>
@@ -7936,7 +7938,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="130" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A130">
         <v>890</v>
       </c>
@@ -7998,7 +8000,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="131" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A131">
         <v>891</v>
       </c>
@@ -8054,7 +8056,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="132" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A132">
         <v>892</v>
       </c>
@@ -8116,7 +8118,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="133" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A133">
         <v>893</v>
       </c>
@@ -8178,7 +8180,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="134" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A134">
         <v>894</v>
       </c>
@@ -8234,7 +8236,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="135" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A135">
         <v>895</v>
       </c>
@@ -8293,7 +8295,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="136" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A136">
         <v>896</v>
       </c>
@@ -8352,7 +8354,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="137" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A137">
         <v>897</v>
       </c>
@@ -8414,7 +8416,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="138" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A138">
         <v>898</v>
       </c>
@@ -8473,7 +8475,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="139" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A139">
         <v>899</v>
       </c>
@@ -8535,7 +8537,7 @@
         <v>-6</v>
       </c>
     </row>
-    <row r="140" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A140">
         <v>900</v>
       </c>
@@ -8588,7 +8590,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="141" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A141">
         <v>901</v>
       </c>
@@ -8644,7 +8646,7 @@
         <v>-6</v>
       </c>
     </row>
-    <row r="142" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A142">
         <v>902</v>
       </c>
@@ -8697,7 +8699,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="143" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A143">
         <v>903</v>
       </c>
@@ -8753,7 +8755,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="144" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A144">
         <v>904</v>
       </c>
@@ -8794,7 +8796,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="145" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A145">
         <v>905</v>
       </c>
@@ -8853,7 +8855,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="146" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A146">
         <v>906</v>
       </c>
@@ -8912,7 +8914,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="147" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A147">
         <v>908</v>
       </c>
@@ -8968,7 +8970,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="148" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A148">
         <v>909</v>
       </c>
@@ -9024,7 +9026,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="149" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A149">
         <v>910</v>
       </c>
@@ -9083,7 +9085,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="150" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A150">
         <v>912</v>
       </c>
@@ -9139,7 +9141,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="151" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A151">
         <v>913</v>
       </c>
@@ -9201,7 +9203,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="152" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A152">
         <v>914</v>
       </c>
@@ -9263,7 +9265,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="153" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A153">
         <v>915</v>
       </c>
@@ -9325,7 +9327,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="154" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A154">
         <v>916</v>
       </c>
@@ -9375,7 +9377,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="155" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A155">
         <v>917</v>
       </c>
@@ -9428,7 +9430,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="156" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A156">
         <v>918</v>
       </c>
@@ -9487,7 +9489,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="157" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A157">
         <v>919</v>
       </c>
@@ -9546,7 +9548,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="158" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A158">
         <v>920</v>
       </c>
@@ -9608,7 +9610,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="159" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A159">
         <v>922</v>
       </c>
@@ -9664,7 +9666,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="160" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A160">
         <v>923</v>
       </c>
@@ -9726,7 +9728,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="161" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A161">
         <v>924</v>
       </c>
@@ -9785,7 +9787,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="162" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A162">
         <v>925</v>
       </c>
@@ -9844,7 +9846,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="163" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A163">
         <v>926</v>
       </c>
@@ -9900,7 +9902,7 @@
         <v>-9</v>
       </c>
     </row>
-    <row r="164" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A164">
         <v>927</v>
       </c>
@@ -9956,7 +9958,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A165">
         <v>928</v>
       </c>
@@ -10018,7 +10020,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="166" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A166">
         <v>929</v>
       </c>
@@ -10080,7 +10082,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="167" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A167">
         <v>930</v>
       </c>
@@ -10130,7 +10132,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="168" spans="1:21" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:21" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A168">
         <v>931</v>
       </c>
@@ -10191,7 +10193,7 @@
       </c>
       <c r="U168"/>
     </row>
-    <row r="169" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A169">
         <v>932</v>
       </c>
@@ -10253,7 +10255,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="170" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A170">
         <v>933</v>
       </c>
@@ -10315,7 +10317,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="171" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A171">
         <v>934</v>
       </c>
@@ -10377,7 +10379,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="172" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A172">
         <v>935</v>
       </c>
@@ -10430,7 +10432,7 @@
         <v>-6</v>
       </c>
     </row>
-    <row r="173" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A173">
         <v>936</v>
       </c>
@@ -10489,7 +10491,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="174" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A174">
         <v>937</v>
       </c>
@@ -10551,7 +10553,7 @@
         <v>-6</v>
       </c>
     </row>
-    <row r="175" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A175">
         <v>938</v>
       </c>
@@ -10613,7 +10615,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="176" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A176">
         <v>939</v>
       </c>
@@ -10672,7 +10674,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="177" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A177">
         <v>941</v>
       </c>
@@ -10734,7 +10736,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A178">
         <v>942</v>
       </c>
@@ -10796,7 +10798,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="179" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A179">
         <v>943</v>
       </c>
@@ -10858,7 +10860,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A180">
         <v>944</v>
       </c>
@@ -10917,7 +10919,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="181" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A181">
         <v>945</v>
       </c>
@@ -10979,7 +10981,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="182" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A182">
         <v>946</v>
       </c>
@@ -11041,7 +11043,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="183" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A183">
         <v>947</v>
       </c>
@@ -11094,7 +11096,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="184" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A184">
         <v>948</v>
       </c>
@@ -11156,7 +11158,7 @@
         <v>-6</v>
       </c>
     </row>
-    <row r="185" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A185">
         <v>949</v>
       </c>
@@ -11203,7 +11205,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="186" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A186">
         <v>950</v>
       </c>
@@ -11259,7 +11261,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="187" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A187">
         <v>951</v>
       </c>
@@ -11321,7 +11323,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="188" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A188">
         <v>952</v>
       </c>
@@ -11383,7 +11385,7 @@
         <v>-6</v>
       </c>
     </row>
-    <row r="189" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A189">
         <v>953</v>
       </c>
@@ -11445,7 +11447,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="190" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A190">
         <v>954</v>
       </c>
@@ -11504,7 +11506,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="191" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A191">
         <v>955</v>
       </c>
@@ -11566,7 +11568,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="192" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A192">
         <v>956</v>
       </c>
@@ -11628,7 +11630,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="193" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A193">
         <v>957</v>
       </c>
@@ -11690,7 +11692,7 @@
         <v>-6</v>
       </c>
     </row>
-    <row r="194" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A194">
         <v>958</v>
       </c>
@@ -11749,7 +11751,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="195" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A195">
         <v>959</v>
       </c>
@@ -11805,7 +11807,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="196" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A196">
         <v>960</v>
       </c>
@@ -11861,7 +11863,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="197" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A197">
         <v>961</v>
       </c>
@@ -11917,7 +11919,7 @@
         <v>-10</v>
       </c>
     </row>
-    <row r="198" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A198">
         <v>962</v>
       </c>
@@ -11979,7 +11981,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="199" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A199">
         <v>963</v>
       </c>
@@ -12032,7 +12034,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="200" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A200">
         <v>964</v>
       </c>
@@ -12094,7 +12096,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="201" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A201">
         <v>966</v>
       </c>
@@ -12153,7 +12155,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="202" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A202">
         <v>967</v>
       </c>
@@ -12206,7 +12208,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="203" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A203">
         <v>968</v>
       </c>
@@ -12268,7 +12270,7 @@
         <v>-8</v>
       </c>
     </row>
-    <row r="204" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A204">
         <v>969</v>
       </c>
@@ -12330,7 +12332,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="205" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A205">
         <v>970</v>
       </c>
@@ -12389,7 +12391,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="206" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A206">
         <v>971</v>
       </c>
@@ -12448,7 +12450,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="207" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A207">
         <v>972</v>
       </c>
@@ -12507,7 +12509,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="208" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A208">
         <v>974</v>
       </c>
@@ -12569,7 +12571,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="209" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A209">
         <v>975</v>
       </c>
@@ -12628,7 +12630,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="210" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A210">
         <v>976</v>
       </c>
@@ -12666,7 +12668,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="211" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A211">
         <v>977</v>
       </c>
@@ -12701,7 +12703,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="212" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A212">
         <v>978</v>
       </c>
@@ -12742,7 +12744,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="213" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A213">
         <v>979</v>
       </c>
@@ -12783,7 +12785,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="214" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A214">
         <v>980</v>
       </c>
@@ -12827,7 +12829,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="215" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A215">
         <v>981</v>
       </c>
@@ -12883,7 +12885,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="216" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A216">
         <v>982</v>
       </c>
@@ -12924,7 +12926,7 @@
         <v>-6</v>
       </c>
     </row>
-    <row r="217" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A217">
         <v>983</v>
       </c>
@@ -12962,7 +12964,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="218" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A218">
         <v>984</v>
       </c>
@@ -13012,7 +13014,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="219" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A219">
         <v>985</v>
       </c>
@@ -13059,7 +13061,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="220" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A220">
         <v>986</v>
       </c>
@@ -13109,7 +13111,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="221" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A221">
         <v>987</v>
       </c>
@@ -13156,7 +13158,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="222" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A222">
         <v>988</v>
       </c>
@@ -13194,7 +13196,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="223" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A223">
         <v>989</v>
       </c>
@@ -13244,7 +13246,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="224" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A224">
         <v>990</v>
       </c>
@@ -13294,7 +13296,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="225" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A225">
         <v>992</v>
       </c>
@@ -13344,7 +13346,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="226" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A226">
         <v>993</v>
       </c>
@@ -13397,7 +13399,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="227" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A227">
         <v>994</v>
       </c>
@@ -13447,7 +13449,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="228" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A228">
         <v>995</v>
       </c>
@@ -13500,7 +13502,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="229" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A229">
         <v>996</v>
       </c>
@@ -13553,7 +13555,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="230" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A230">
         <v>997</v>
       </c>
@@ -13588,7 +13590,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="231" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A231">
         <v>998</v>
       </c>
@@ -13629,7 +13631,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="232" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A232">
         <v>999</v>
       </c>
@@ -13682,7 +13684,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="233" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A233">
         <v>1000</v>
       </c>
@@ -13726,7 +13728,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="234" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A234">
         <v>1001</v>
       </c>
@@ -13776,7 +13778,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="235" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A235">
         <v>1002</v>
       </c>
@@ -13814,7 +13816,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="236" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A236">
         <v>1003</v>
       </c>
@@ -13870,7 +13872,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="237" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A237">
         <v>1004</v>
       </c>
@@ -13929,7 +13931,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="238" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A238">
         <v>1005</v>
       </c>
@@ -13985,7 +13987,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="239" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A239">
         <v>1006</v>
       </c>
@@ -14029,7 +14031,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="240" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A240">
         <v>1007</v>
       </c>
@@ -14079,7 +14081,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="241" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A241">
         <v>1008</v>
       </c>
@@ -14138,7 +14140,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="242" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A242">
         <v>1009</v>
       </c>
@@ -14191,7 +14193,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="243" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A243">
         <v>1010</v>
       </c>
@@ -14244,7 +14246,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="244" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A244">
         <v>1011</v>
       </c>
@@ -14303,7 +14305,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="245" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A245">
         <v>1012</v>
       </c>
@@ -14362,7 +14364,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="246" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A246">
         <v>1013</v>
       </c>
@@ -14424,7 +14426,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="247" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A247">
         <v>1014</v>
       </c>
@@ -14480,7 +14482,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="248" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A248">
         <v>1015</v>
       </c>
@@ -14530,7 +14532,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="249" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A249">
         <v>1016</v>
       </c>
@@ -14589,7 +14591,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="250" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A250">
         <v>1017</v>
       </c>
@@ -14651,7 +14653,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="251" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A251">
         <v>1018</v>
       </c>
@@ -14713,7 +14715,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="252" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A252">
         <v>1019</v>
       </c>
@@ -14772,7 +14774,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="253" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A253">
         <v>1020</v>
       </c>
@@ -14834,7 +14836,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="254" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A254">
         <v>1021</v>
       </c>
@@ -14893,7 +14895,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="255" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A255">
         <v>1022</v>
       </c>
@@ -14940,7 +14942,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="256" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A256">
         <v>1023</v>
       </c>
@@ -14981,7 +14983,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="257" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A257">
         <v>1024</v>
       </c>
@@ -15034,7 +15036,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="258" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A258">
         <v>1025</v>
       </c>
@@ -15084,7 +15086,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="259" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A259">
         <v>1026</v>
       </c>
@@ -15134,7 +15136,7 @@
         <v>-6</v>
       </c>
     </row>
-    <row r="260" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A260">
         <v>1027</v>
       </c>
@@ -15178,7 +15180,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="261" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A261">
         <v>1028</v>
       </c>
@@ -15219,7 +15221,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="262" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A262">
         <v>1029</v>
       </c>
@@ -15269,7 +15271,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="263" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A263">
         <v>1030</v>
       </c>
@@ -15325,7 +15327,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="264" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A264">
         <v>1031</v>
       </c>
@@ -15381,7 +15383,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="265" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A265">
         <v>1032</v>
       </c>
@@ -15425,7 +15427,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="266" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A266">
         <v>1033</v>
       </c>
@@ -15458,6 +15460,53 @@
       </c>
       <c r="U266">
         <v>2</v>
+      </c>
+    </row>
+    <row r="267" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="B267">
+        <v>221</v>
+      </c>
+      <c r="C267">
+        <v>5</v>
+      </c>
+      <c r="E267">
+        <v>13703</v>
+      </c>
+      <c r="F267">
+        <v>19805</v>
+      </c>
+      <c r="G267">
+        <v>12235</v>
+      </c>
+      <c r="H267">
+        <v>19999</v>
+      </c>
+      <c r="I267">
+        <v>20558</v>
+      </c>
+      <c r="J267">
+        <v>20728</v>
+      </c>
+      <c r="N267">
+        <v>4</v>
+      </c>
+      <c r="O267">
+        <v>4</v>
+      </c>
+      <c r="Q267">
+        <v>7</v>
+      </c>
+      <c r="R267">
+        <v>4</v>
+      </c>
+      <c r="S267">
+        <v>0</v>
+      </c>
+      <c r="U267">
+        <v>3</v>
+      </c>
+      <c r="V267">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -15468,14 +15517,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02C51864-C654-4966-AD8D-26F85A24E18C}">
   <dimension ref="A1:E20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.85546875" customWidth="1"/>
+    <col min="1" max="1" width="13.88671875" customWidth="1"/>
     <col min="2" max="2" width="45" customWidth="1"/>
-    <col min="4" max="4" width="15.85546875" customWidth="1"/>
+    <col min="4" max="4" width="15.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -15486,7 +15535,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -15500,7 +15549,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -15514,7 +15563,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -15528,7 +15577,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -15542,7 +15591,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -15553,7 +15602,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -15564,7 +15613,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -15575,7 +15624,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -15583,7 +15632,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -15591,7 +15640,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -15599,7 +15648,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -15607,7 +15656,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -15615,7 +15664,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -15623,7 +15672,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>14</v>
       </c>
@@ -15631,7 +15680,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>15</v>
       </c>
@@ -15639,7 +15688,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>16</v>
       </c>
@@ -15647,7 +15696,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>17</v>
       </c>
@@ -15655,7 +15704,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>18</v>
       </c>
@@ -15663,7 +15712,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>19</v>
       </c>

</xml_diff>

<commit_message>
should officially have newest data updated
</commit_message>
<xml_diff>
--- a/datasets/xlsx/CSPreMatchStatistics.xlsx
+++ b/datasets/xlsx/CSPreMatchStatistics.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexPost\repos\HardWareWebsite\datasets\xlsx\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexPost\Repos\HardWareWebsite\datasets\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B12050F-519B-4520-A506-AF3D151ADA60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FAF4F72-48CA-4A90-AE91-A8935952CE0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -477,28 +477,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V267"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:V268"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="14.88671875" customWidth="1"/>
-    <col min="3" max="3" width="13.33203125" customWidth="1"/>
-    <col min="4" max="5" width="13.5546875" customWidth="1"/>
-    <col min="6" max="6" width="12.33203125" customWidth="1"/>
+    <col min="2" max="2" width="14.85546875" customWidth="1"/>
+    <col min="3" max="3" width="13.28515625" customWidth="1"/>
+    <col min="4" max="5" width="13.5703125" customWidth="1"/>
+    <col min="6" max="6" width="12.28515625" customWidth="1"/>
     <col min="7" max="7" width="12" customWidth="1"/>
-    <col min="8" max="8" width="12.5546875" customWidth="1"/>
-    <col min="9" max="9" width="11.33203125" customWidth="1"/>
-    <col min="10" max="10" width="10.5546875" customWidth="1"/>
+    <col min="8" max="8" width="12.5703125" customWidth="1"/>
+    <col min="9" max="9" width="11.28515625" customWidth="1"/>
+    <col min="10" max="10" width="10.5703125" customWidth="1"/>
     <col min="11" max="11" width="11" customWidth="1"/>
-    <col min="12" max="13" width="10.44140625" customWidth="1"/>
-    <col min="14" max="14" width="11.5546875" customWidth="1"/>
-    <col min="15" max="15" width="10.44140625" customWidth="1"/>
-    <col min="17" max="17" width="9.5546875" customWidth="1"/>
-    <col min="19" max="19" width="11.6640625" customWidth="1"/>
-    <col min="20" max="20" width="12.88671875" customWidth="1"/>
-    <col min="21" max="21" width="11.44140625" customWidth="1"/>
+    <col min="12" max="13" width="10.42578125" customWidth="1"/>
+    <col min="14" max="14" width="11.5703125" customWidth="1"/>
+    <col min="15" max="15" width="10.42578125" customWidth="1"/>
+    <col min="17" max="17" width="9.5703125" customWidth="1"/>
+    <col min="19" max="19" width="11.7109375" customWidth="1"/>
+    <col min="20" max="20" width="12.85546875" customWidth="1"/>
+    <col min="21" max="21" width="11.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -566,7 +566,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>744</v>
       </c>
@@ -610,7 +610,7 @@
         <v>-6</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>745</v>
       </c>
@@ -651,7 +651,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>750</v>
       </c>
@@ -701,7 +701,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>752</v>
       </c>
@@ -757,7 +757,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>753</v>
       </c>
@@ -816,7 +816,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>754</v>
       </c>
@@ -872,7 +872,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>755</v>
       </c>
@@ -928,7 +928,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>756</v>
       </c>
@@ -984,7 +984,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>757</v>
       </c>
@@ -1028,7 +1028,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>758</v>
       </c>
@@ -1069,7 +1069,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>759</v>
       </c>
@@ -1122,7 +1122,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>760</v>
       </c>
@@ -1178,7 +1178,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>761</v>
       </c>
@@ -1240,7 +1240,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>762</v>
       </c>
@@ -1293,7 +1293,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>763</v>
       </c>
@@ -1349,7 +1349,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>764</v>
       </c>
@@ -1408,7 +1408,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>765</v>
       </c>
@@ -1458,7 +1458,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>766</v>
       </c>
@@ -1502,7 +1502,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>767</v>
       </c>
@@ -1561,7 +1561,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>768</v>
       </c>
@@ -1617,7 +1617,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>769</v>
       </c>
@@ -1679,7 +1679,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>770</v>
       </c>
@@ -1738,7 +1738,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>771</v>
       </c>
@@ -1791,7 +1791,7 @@
         <v>-6</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>772</v>
       </c>
@@ -1838,7 +1838,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>773</v>
       </c>
@@ -1894,7 +1894,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>775</v>
       </c>
@@ -1953,7 +1953,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>776</v>
       </c>
@@ -2009,7 +2009,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>777</v>
       </c>
@@ -2071,7 +2071,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>780</v>
       </c>
@@ -2133,7 +2133,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>781</v>
       </c>
@@ -2192,7 +2192,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>782</v>
       </c>
@@ -2251,7 +2251,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>783</v>
       </c>
@@ -2310,7 +2310,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="34" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>784</v>
       </c>
@@ -2369,7 +2369,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="35" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>785</v>
       </c>
@@ -2428,7 +2428,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="36" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>786</v>
       </c>
@@ -2490,7 +2490,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="37" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>787</v>
       </c>
@@ -2546,7 +2546,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="38" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>788</v>
       </c>
@@ -2593,7 +2593,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="39" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>789</v>
       </c>
@@ -2649,7 +2649,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="40" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>790</v>
       </c>
@@ -2705,7 +2705,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="41" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>791</v>
       </c>
@@ -2761,7 +2761,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="42" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>792</v>
       </c>
@@ -2823,7 +2823,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="43" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>793</v>
       </c>
@@ -2885,7 +2885,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="44" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>794</v>
       </c>
@@ -2947,7 +2947,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="45" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>795</v>
       </c>
@@ -3006,7 +3006,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>796</v>
       </c>
@@ -3068,7 +3068,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="47" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>797</v>
       </c>
@@ -3124,7 +3124,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="48" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>798</v>
       </c>
@@ -3180,7 +3180,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="49" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>799</v>
       </c>
@@ -3233,7 +3233,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>800</v>
       </c>
@@ -3295,7 +3295,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="51" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>801</v>
       </c>
@@ -3354,7 +3354,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>802</v>
       </c>
@@ -3407,7 +3407,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="53" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>803</v>
       </c>
@@ -3460,7 +3460,7 @@
         <v>-13</v>
       </c>
     </row>
-    <row r="54" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>804</v>
       </c>
@@ -3522,7 +3522,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="55" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>805</v>
       </c>
@@ -3578,7 +3578,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="56" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>807</v>
       </c>
@@ -3631,7 +3631,7 @@
         <v>-8</v>
       </c>
     </row>
-    <row r="57" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>808</v>
       </c>
@@ -3687,7 +3687,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="58" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>809</v>
       </c>
@@ -3749,7 +3749,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="59" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>810</v>
       </c>
@@ -3808,7 +3808,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="60" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>811</v>
       </c>
@@ -3870,7 +3870,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="61" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>812</v>
       </c>
@@ -3929,7 +3929,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>813</v>
       </c>
@@ -3988,7 +3988,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="63" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>814</v>
       </c>
@@ -4044,7 +4044,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="64" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>815</v>
       </c>
@@ -4100,7 +4100,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="65" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>818</v>
       </c>
@@ -4147,7 +4147,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>819</v>
       </c>
@@ -4200,7 +4200,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="67" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>820</v>
       </c>
@@ -4259,7 +4259,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="68" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>821</v>
       </c>
@@ -4318,7 +4318,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="69" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>822</v>
       </c>
@@ -4374,7 +4374,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="70" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>823</v>
       </c>
@@ -4424,7 +4424,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="71" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>824</v>
       </c>
@@ -4483,7 +4483,7 @@
         <v>-6</v>
       </c>
     </row>
-    <row r="72" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>826</v>
       </c>
@@ -4542,7 +4542,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="73" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>827</v>
       </c>
@@ -4604,7 +4604,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>828</v>
       </c>
@@ -4660,7 +4660,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="75" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>830</v>
       </c>
@@ -4722,7 +4722,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>831</v>
       </c>
@@ -4778,7 +4778,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="77" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>832</v>
       </c>
@@ -4831,7 +4831,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="78" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>833</v>
       </c>
@@ -4893,7 +4893,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="79" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>834</v>
       </c>
@@ -4949,7 +4949,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="80" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>835</v>
       </c>
@@ -5011,7 +5011,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="81" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>836</v>
       </c>
@@ -5073,7 +5073,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="82" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>837</v>
       </c>
@@ -5135,7 +5135,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="83" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>838</v>
       </c>
@@ -5197,7 +5197,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="84" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>839</v>
       </c>
@@ -5256,7 +5256,7 @@
         <v>-8</v>
       </c>
     </row>
-    <row r="85" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>840</v>
       </c>
@@ -5318,7 +5318,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="86" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>841</v>
       </c>
@@ -5374,7 +5374,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="87" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>842</v>
       </c>
@@ -5433,7 +5433,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="88" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>843</v>
       </c>
@@ -5495,7 +5495,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="89" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>844</v>
       </c>
@@ -5551,7 +5551,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>845</v>
       </c>
@@ -5613,7 +5613,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="91" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>846</v>
       </c>
@@ -5672,7 +5672,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="92" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>848</v>
       </c>
@@ -5734,7 +5734,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="93" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>850</v>
       </c>
@@ -5796,7 +5796,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="94" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>851</v>
       </c>
@@ -5855,7 +5855,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="95" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>853</v>
       </c>
@@ -5917,7 +5917,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="96" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>854</v>
       </c>
@@ -5976,7 +5976,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="97" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>855</v>
       </c>
@@ -6032,7 +6032,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="98" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>856</v>
       </c>
@@ -6094,7 +6094,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="99" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>857</v>
       </c>
@@ -6150,7 +6150,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>859</v>
       </c>
@@ -6212,7 +6212,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="101" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>860</v>
       </c>
@@ -6274,7 +6274,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="102" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>861</v>
       </c>
@@ -6333,7 +6333,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="103" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>862</v>
       </c>
@@ -6392,7 +6392,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="104" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>863</v>
       </c>
@@ -6454,7 +6454,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="105" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>864</v>
       </c>
@@ -6516,7 +6516,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="106" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>865</v>
       </c>
@@ -6575,7 +6575,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="107" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>866</v>
       </c>
@@ -6634,7 +6634,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="108" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>867</v>
       </c>
@@ -6693,7 +6693,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="109" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>868</v>
       </c>
@@ -6752,7 +6752,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="110" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>869</v>
       </c>
@@ -6814,7 +6814,7 @@
         <v>-9</v>
       </c>
     </row>
-    <row r="111" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>870</v>
       </c>
@@ -6876,7 +6876,7 @@
         <v>-9</v>
       </c>
     </row>
-    <row r="112" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>871</v>
       </c>
@@ -6935,7 +6935,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="113" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>872</v>
       </c>
@@ -6997,7 +6997,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="114" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>873</v>
       </c>
@@ -7056,7 +7056,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="115" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>874</v>
       </c>
@@ -7115,7 +7115,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>875</v>
       </c>
@@ -7174,7 +7174,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="117" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>876</v>
       </c>
@@ -7236,7 +7236,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="118" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>877</v>
       </c>
@@ -7298,7 +7298,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="119" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>878</v>
       </c>
@@ -7357,7 +7357,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="120" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>880</v>
       </c>
@@ -7419,7 +7419,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>881</v>
       </c>
@@ -7478,7 +7478,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="122" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>882</v>
       </c>
@@ -7537,7 +7537,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="123" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A123">
         <v>883</v>
       </c>
@@ -7599,7 +7599,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="124" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A124">
         <v>884</v>
       </c>
@@ -7646,7 +7646,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="125" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A125">
         <v>885</v>
       </c>
@@ -7705,7 +7705,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="126" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A126">
         <v>886</v>
       </c>
@@ -7764,7 +7764,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="127" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>887</v>
       </c>
@@ -7820,7 +7820,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>888</v>
       </c>
@@ -7879,7 +7879,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="129" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A129">
         <v>889</v>
       </c>
@@ -7938,7 +7938,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="130" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A130">
         <v>890</v>
       </c>
@@ -8000,7 +8000,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="131" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A131">
         <v>891</v>
       </c>
@@ -8056,7 +8056,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="132" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A132">
         <v>892</v>
       </c>
@@ -8118,7 +8118,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="133" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A133">
         <v>893</v>
       </c>
@@ -8180,7 +8180,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="134" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A134">
         <v>894</v>
       </c>
@@ -8236,7 +8236,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="135" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A135">
         <v>895</v>
       </c>
@@ -8295,7 +8295,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="136" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A136">
         <v>896</v>
       </c>
@@ -8354,7 +8354,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="137" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A137">
         <v>897</v>
       </c>
@@ -8416,7 +8416,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="138" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A138">
         <v>898</v>
       </c>
@@ -8475,7 +8475,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="139" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A139">
         <v>899</v>
       </c>
@@ -8537,7 +8537,7 @@
         <v>-6</v>
       </c>
     </row>
-    <row r="140" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A140">
         <v>900</v>
       </c>
@@ -8590,7 +8590,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="141" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A141">
         <v>901</v>
       </c>
@@ -8646,7 +8646,7 @@
         <v>-6</v>
       </c>
     </row>
-    <row r="142" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A142">
         <v>902</v>
       </c>
@@ -8699,7 +8699,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="143" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A143">
         <v>903</v>
       </c>
@@ -8755,7 +8755,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="144" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A144">
         <v>904</v>
       </c>
@@ -8796,7 +8796,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="145" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A145">
         <v>905</v>
       </c>
@@ -8855,7 +8855,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="146" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A146">
         <v>906</v>
       </c>
@@ -8914,7 +8914,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="147" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A147">
         <v>908</v>
       </c>
@@ -8970,7 +8970,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="148" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A148">
         <v>909</v>
       </c>
@@ -9026,7 +9026,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="149" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A149">
         <v>910</v>
       </c>
@@ -9085,7 +9085,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="150" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A150">
         <v>912</v>
       </c>
@@ -9141,7 +9141,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="151" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A151">
         <v>913</v>
       </c>
@@ -9203,7 +9203,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="152" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A152">
         <v>914</v>
       </c>
@@ -9265,7 +9265,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="153" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A153">
         <v>915</v>
       </c>
@@ -9327,7 +9327,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="154" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A154">
         <v>916</v>
       </c>
@@ -9377,7 +9377,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="155" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A155">
         <v>917</v>
       </c>
@@ -9430,7 +9430,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="156" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A156">
         <v>918</v>
       </c>
@@ -9489,7 +9489,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="157" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A157">
         <v>919</v>
       </c>
@@ -9548,7 +9548,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="158" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A158">
         <v>920</v>
       </c>
@@ -9610,7 +9610,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="159" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A159">
         <v>922</v>
       </c>
@@ -9666,7 +9666,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="160" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A160">
         <v>923</v>
       </c>
@@ -9728,7 +9728,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="161" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A161">
         <v>924</v>
       </c>
@@ -9787,7 +9787,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="162" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A162">
         <v>925</v>
       </c>
@@ -9846,7 +9846,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="163" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A163">
         <v>926</v>
       </c>
@@ -9902,7 +9902,7 @@
         <v>-9</v>
       </c>
     </row>
-    <row r="164" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A164">
         <v>927</v>
       </c>
@@ -9958,7 +9958,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A165">
         <v>928</v>
       </c>
@@ -10020,7 +10020,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="166" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A166">
         <v>929</v>
       </c>
@@ -10082,7 +10082,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="167" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A167">
         <v>930</v>
       </c>
@@ -10132,7 +10132,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="168" spans="1:21" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:21" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A168">
         <v>931</v>
       </c>
@@ -10193,7 +10193,7 @@
       </c>
       <c r="U168"/>
     </row>
-    <row r="169" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A169">
         <v>932</v>
       </c>
@@ -10255,7 +10255,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="170" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A170">
         <v>933</v>
       </c>
@@ -10317,7 +10317,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="171" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A171">
         <v>934</v>
       </c>
@@ -10379,7 +10379,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="172" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A172">
         <v>935</v>
       </c>
@@ -10432,7 +10432,7 @@
         <v>-6</v>
       </c>
     </row>
-    <row r="173" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A173">
         <v>936</v>
       </c>
@@ -10491,7 +10491,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="174" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A174">
         <v>937</v>
       </c>
@@ -10553,7 +10553,7 @@
         <v>-6</v>
       </c>
     </row>
-    <row r="175" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A175">
         <v>938</v>
       </c>
@@ -10615,7 +10615,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="176" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A176">
         <v>939</v>
       </c>
@@ -10674,7 +10674,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="177" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A177">
         <v>941</v>
       </c>
@@ -10736,7 +10736,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A178">
         <v>942</v>
       </c>
@@ -10798,7 +10798,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="179" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A179">
         <v>943</v>
       </c>
@@ -10860,7 +10860,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A180">
         <v>944</v>
       </c>
@@ -10919,7 +10919,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="181" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A181">
         <v>945</v>
       </c>
@@ -10981,7 +10981,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="182" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A182">
         <v>946</v>
       </c>
@@ -11043,7 +11043,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="183" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A183">
         <v>947</v>
       </c>
@@ -11096,7 +11096,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="184" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A184">
         <v>948</v>
       </c>
@@ -11158,7 +11158,7 @@
         <v>-6</v>
       </c>
     </row>
-    <row r="185" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A185">
         <v>949</v>
       </c>
@@ -11205,7 +11205,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="186" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A186">
         <v>950</v>
       </c>
@@ -11261,7 +11261,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="187" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A187">
         <v>951</v>
       </c>
@@ -11323,7 +11323,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="188" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A188">
         <v>952</v>
       </c>
@@ -11385,7 +11385,7 @@
         <v>-6</v>
       </c>
     </row>
-    <row r="189" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A189">
         <v>953</v>
       </c>
@@ -11447,7 +11447,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="190" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A190">
         <v>954</v>
       </c>
@@ -11506,7 +11506,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="191" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A191">
         <v>955</v>
       </c>
@@ -11568,7 +11568,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="192" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A192">
         <v>956</v>
       </c>
@@ -11630,7 +11630,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="193" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A193">
         <v>957</v>
       </c>
@@ -11692,7 +11692,7 @@
         <v>-6</v>
       </c>
     </row>
-    <row r="194" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A194">
         <v>958</v>
       </c>
@@ -11751,7 +11751,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="195" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A195">
         <v>959</v>
       </c>
@@ -11807,7 +11807,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="196" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A196">
         <v>960</v>
       </c>
@@ -11863,7 +11863,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="197" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A197">
         <v>961</v>
       </c>
@@ -11919,7 +11919,7 @@
         <v>-10</v>
       </c>
     </row>
-    <row r="198" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A198">
         <v>962</v>
       </c>
@@ -11981,7 +11981,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="199" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A199">
         <v>963</v>
       </c>
@@ -12034,7 +12034,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="200" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A200">
         <v>964</v>
       </c>
@@ -12096,7 +12096,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="201" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A201">
         <v>966</v>
       </c>
@@ -12155,7 +12155,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="202" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A202">
         <v>967</v>
       </c>
@@ -12208,7 +12208,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="203" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A203">
         <v>968</v>
       </c>
@@ -12270,7 +12270,7 @@
         <v>-8</v>
       </c>
     </row>
-    <row r="204" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A204">
         <v>969</v>
       </c>
@@ -12332,7 +12332,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="205" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A205">
         <v>970</v>
       </c>
@@ -12391,7 +12391,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="206" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A206">
         <v>971</v>
       </c>
@@ -12450,7 +12450,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="207" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A207">
         <v>972</v>
       </c>
@@ -12509,7 +12509,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="208" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A208">
         <v>974</v>
       </c>
@@ -12571,7 +12571,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="209" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A209">
         <v>975</v>
       </c>
@@ -12630,7 +12630,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="210" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A210">
         <v>976</v>
       </c>
@@ -12668,7 +12668,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="211" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A211">
         <v>977</v>
       </c>
@@ -12703,7 +12703,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="212" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A212">
         <v>978</v>
       </c>
@@ -12744,7 +12744,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="213" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A213">
         <v>979</v>
       </c>
@@ -12785,7 +12785,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="214" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A214">
         <v>980</v>
       </c>
@@ -12829,7 +12829,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="215" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A215">
         <v>981</v>
       </c>
@@ -12885,7 +12885,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="216" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A216">
         <v>982</v>
       </c>
@@ -12926,7 +12926,7 @@
         <v>-6</v>
       </c>
     </row>
-    <row r="217" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A217">
         <v>983</v>
       </c>
@@ -12964,7 +12964,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="218" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A218">
         <v>984</v>
       </c>
@@ -13014,7 +13014,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="219" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A219">
         <v>985</v>
       </c>
@@ -13061,7 +13061,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="220" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A220">
         <v>986</v>
       </c>
@@ -13111,7 +13111,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="221" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A221">
         <v>987</v>
       </c>
@@ -13158,7 +13158,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="222" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A222">
         <v>988</v>
       </c>
@@ -13196,7 +13196,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="223" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A223">
         <v>989</v>
       </c>
@@ -13246,7 +13246,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="224" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A224">
         <v>990</v>
       </c>
@@ -13296,7 +13296,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="225" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A225">
         <v>992</v>
       </c>
@@ -13346,7 +13346,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="226" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A226">
         <v>993</v>
       </c>
@@ -13399,7 +13399,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="227" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A227">
         <v>994</v>
       </c>
@@ -13449,7 +13449,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="228" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A228">
         <v>995</v>
       </c>
@@ -13502,7 +13502,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="229" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A229">
         <v>996</v>
       </c>
@@ -13555,7 +13555,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="230" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A230">
         <v>997</v>
       </c>
@@ -13590,7 +13590,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="231" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A231">
         <v>998</v>
       </c>
@@ -13631,7 +13631,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="232" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A232">
         <v>999</v>
       </c>
@@ -13684,7 +13684,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="233" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A233">
         <v>1000</v>
       </c>
@@ -13728,7 +13728,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="234" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A234">
         <v>1001</v>
       </c>
@@ -13778,7 +13778,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="235" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A235">
         <v>1002</v>
       </c>
@@ -13816,7 +13816,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="236" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A236">
         <v>1003</v>
       </c>
@@ -13872,7 +13872,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="237" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A237">
         <v>1004</v>
       </c>
@@ -13931,7 +13931,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="238" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A238">
         <v>1005</v>
       </c>
@@ -13987,7 +13987,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="239" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A239">
         <v>1006</v>
       </c>
@@ -14031,7 +14031,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="240" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A240">
         <v>1007</v>
       </c>
@@ -14081,7 +14081,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="241" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A241">
         <v>1008</v>
       </c>
@@ -14140,7 +14140,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="242" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A242">
         <v>1009</v>
       </c>
@@ -14193,7 +14193,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="243" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A243">
         <v>1010</v>
       </c>
@@ -14246,7 +14246,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="244" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A244">
         <v>1011</v>
       </c>
@@ -14305,7 +14305,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="245" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A245">
         <v>1012</v>
       </c>
@@ -14364,7 +14364,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="246" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A246">
         <v>1013</v>
       </c>
@@ -14426,7 +14426,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="247" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A247">
         <v>1014</v>
       </c>
@@ -14482,7 +14482,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="248" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A248">
         <v>1015</v>
       </c>
@@ -14532,7 +14532,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="249" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A249">
         <v>1016</v>
       </c>
@@ -14591,7 +14591,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="250" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A250">
         <v>1017</v>
       </c>
@@ -14653,7 +14653,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="251" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A251">
         <v>1018</v>
       </c>
@@ -14715,7 +14715,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="252" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A252">
         <v>1019</v>
       </c>
@@ -14774,7 +14774,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="253" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A253">
         <v>1020</v>
       </c>
@@ -14836,7 +14836,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="254" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A254">
         <v>1021</v>
       </c>
@@ -14895,7 +14895,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="255" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A255">
         <v>1022</v>
       </c>
@@ -14942,7 +14942,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="256" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A256">
         <v>1023</v>
       </c>
@@ -14983,7 +14983,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="257" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A257">
         <v>1024</v>
       </c>
@@ -15036,7 +15036,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="258" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A258">
         <v>1025</v>
       </c>
@@ -15086,7 +15086,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="259" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A259">
         <v>1026</v>
       </c>
@@ -15136,7 +15136,7 @@
         <v>-6</v>
       </c>
     </row>
-    <row r="260" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A260">
         <v>1027</v>
       </c>
@@ -15180,7 +15180,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="261" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A261">
         <v>1028</v>
       </c>
@@ -15221,7 +15221,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="262" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A262">
         <v>1029</v>
       </c>
@@ -15271,7 +15271,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="263" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A263">
         <v>1030</v>
       </c>
@@ -15327,7 +15327,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="264" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A264">
         <v>1031</v>
       </c>
@@ -15383,7 +15383,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="265" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A265">
         <v>1032</v>
       </c>
@@ -15427,7 +15427,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="266" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A266">
         <v>1033</v>
       </c>
@@ -15462,7 +15462,10 @@
         <v>2</v>
       </c>
     </row>
-    <row r="267" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A267">
+        <v>1156</v>
+      </c>
       <c r="B267">
         <v>221</v>
       </c>
@@ -15507,6 +15510,59 @@
       </c>
       <c r="V267">
         <v>3</v>
+      </c>
+    </row>
+    <row r="268" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A268">
+        <v>1157</v>
+      </c>
+      <c r="B268">
+        <v>221</v>
+      </c>
+      <c r="C268">
+        <v>311</v>
+      </c>
+      <c r="E268">
+        <v>12341</v>
+      </c>
+      <c r="F268">
+        <v>5212</v>
+      </c>
+      <c r="I268">
+        <v>9498</v>
+      </c>
+      <c r="J268">
+        <v>6447</v>
+      </c>
+      <c r="K268">
+        <v>1191</v>
+      </c>
+      <c r="L268">
+        <v>8139</v>
+      </c>
+      <c r="M268">
+        <v>8437</v>
+      </c>
+      <c r="N268">
+        <v>-6</v>
+      </c>
+      <c r="O268">
+        <v>-11</v>
+      </c>
+      <c r="Q268">
+        <v>-4</v>
+      </c>
+      <c r="R268">
+        <v>3</v>
+      </c>
+      <c r="S268">
+        <v>-5</v>
+      </c>
+      <c r="U268">
+        <v>0</v>
+      </c>
+      <c r="V268">
+        <v>-7</v>
       </c>
     </row>
   </sheetData>
@@ -15517,14 +15573,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02C51864-C654-4966-AD8D-26F85A24E18C}">
   <dimension ref="A1:E20"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.88671875" customWidth="1"/>
+    <col min="1" max="1" width="13.85546875" customWidth="1"/>
     <col min="2" max="2" width="45" customWidth="1"/>
-    <col min="4" max="4" width="15.88671875" customWidth="1"/>
+    <col min="4" max="4" width="15.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -15535,7 +15591,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -15549,7 +15605,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -15563,7 +15619,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -15577,7 +15633,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -15591,7 +15647,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -15602,7 +15658,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -15613,7 +15669,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -15624,7 +15680,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -15632,7 +15688,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -15640,7 +15696,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -15648,7 +15704,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -15656,7 +15712,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -15664,7 +15720,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -15672,7 +15728,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>14</v>
       </c>
@@ -15680,7 +15736,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>15</v>
       </c>
@@ -15688,7 +15744,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>16</v>
       </c>
@@ -15696,7 +15752,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>17</v>
       </c>
@@ -15704,7 +15760,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>18</v>
       </c>
@@ -15712,7 +15768,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>19</v>
       </c>

</xml_diff>

<commit_message>
updated the data here as well lol
</commit_message>
<xml_diff>
--- a/datasets/xlsx/CSPreMatchStatistics.xlsx
+++ b/datasets/xlsx/CSPreMatchStatistics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexPost\Repos\HardWareWebsite\datasets\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FAF4F72-48CA-4A90-AE91-A8935952CE0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FBE0DE4-78F1-4436-94B4-72F162D04EBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -477,7 +477,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V268"/>
+  <dimension ref="A1:V271"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="14.85546875" customWidth="1"/>
@@ -15565,6 +15565,189 @@
         <v>-7</v>
       </c>
     </row>
+    <row r="269" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A269">
+        <v>1158</v>
+      </c>
+      <c r="B269">
+        <v>221</v>
+      </c>
+      <c r="C269">
+        <v>2111</v>
+      </c>
+      <c r="D269">
+        <v>17651</v>
+      </c>
+      <c r="E269">
+        <v>21097</v>
+      </c>
+      <c r="F269">
+        <v>14999</v>
+      </c>
+      <c r="G269">
+        <v>20506</v>
+      </c>
+      <c r="H269">
+        <v>15079</v>
+      </c>
+      <c r="I269">
+        <v>21700</v>
+      </c>
+      <c r="J269">
+        <v>14777</v>
+      </c>
+      <c r="K269">
+        <v>18268</v>
+      </c>
+      <c r="L269">
+        <v>18210</v>
+      </c>
+      <c r="M269">
+        <v>17852</v>
+      </c>
+      <c r="N269">
+        <v>0</v>
+      </c>
+      <c r="O269">
+        <v>4</v>
+      </c>
+      <c r="Q269">
+        <v>1</v>
+      </c>
+      <c r="R269">
+        <v>-7</v>
+      </c>
+      <c r="S269">
+        <v>0</v>
+      </c>
+      <c r="U269">
+        <v>3</v>
+      </c>
+      <c r="V269">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="270" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A270">
+        <v>1159</v>
+      </c>
+      <c r="B270">
+        <v>2111</v>
+      </c>
+      <c r="C270">
+        <v>311</v>
+      </c>
+      <c r="D270">
+        <v>19665</v>
+      </c>
+      <c r="E270">
+        <v>19677</v>
+      </c>
+      <c r="F270">
+        <v>18119</v>
+      </c>
+      <c r="G270">
+        <v>19774</v>
+      </c>
+      <c r="H270">
+        <v>18730</v>
+      </c>
+      <c r="I270">
+        <v>21779</v>
+      </c>
+      <c r="K270">
+        <v>20000</v>
+      </c>
+      <c r="L270">
+        <v>19243</v>
+      </c>
+      <c r="M270">
+        <v>18763</v>
+      </c>
+      <c r="N270">
+        <v>6</v>
+      </c>
+      <c r="O270">
+        <v>-6</v>
+      </c>
+      <c r="Q270">
+        <v>0</v>
+      </c>
+      <c r="R270">
+        <v>2</v>
+      </c>
+      <c r="S270">
+        <v>7</v>
+      </c>
+      <c r="U270">
+        <v>0</v>
+      </c>
+      <c r="V270">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="271" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A271">
+        <v>1160</v>
+      </c>
+      <c r="B271">
+        <v>2111</v>
+      </c>
+      <c r="C271">
+        <v>32</v>
+      </c>
+      <c r="D271">
+        <v>19897</v>
+      </c>
+      <c r="E271">
+        <v>18005</v>
+      </c>
+      <c r="F271">
+        <v>21772</v>
+      </c>
+      <c r="G271">
+        <v>14895</v>
+      </c>
+      <c r="H271">
+        <v>18758</v>
+      </c>
+      <c r="I271">
+        <v>19142</v>
+      </c>
+      <c r="J271">
+        <v>19345</v>
+      </c>
+      <c r="K271">
+        <v>15743</v>
+      </c>
+      <c r="L271">
+        <v>16213</v>
+      </c>
+      <c r="M271">
+        <v>20962</v>
+      </c>
+      <c r="N271">
+        <v>2</v>
+      </c>
+      <c r="O271">
+        <v>-2</v>
+      </c>
+      <c r="Q271">
+        <v>-1</v>
+      </c>
+      <c r="R271">
+        <v>-4</v>
+      </c>
+      <c r="S271">
+        <v>3</v>
+      </c>
+      <c r="U271">
+        <v>-2</v>
+      </c>
+      <c r="V271">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
updated the prematch data
</commit_message>
<xml_diff>
--- a/datasets/xlsx/CSPreMatchStatistics.xlsx
+++ b/datasets/xlsx/CSPreMatchStatistics.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexPost\Repos\HardWareWebsite\datasets\xlsx\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexPost\repos\HardWareWebsite\datasets\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FBE0DE4-78F1-4436-94B4-72F162D04EBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1A83168-879A-454B-800E-3CEBE1F01758}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -477,7 +477,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V271"/>
+  <dimension ref="A1:V272"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="14.85546875" customWidth="1"/>
@@ -15748,6 +15748,68 @@
         <v>4</v>
       </c>
     </row>
+    <row r="272" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A272">
+        <v>1162</v>
+      </c>
+      <c r="B272">
+        <v>32</v>
+      </c>
+      <c r="C272">
+        <v>41</v>
+      </c>
+      <c r="D272">
+        <v>19077</v>
+      </c>
+      <c r="E272">
+        <v>18456</v>
+      </c>
+      <c r="F272">
+        <v>22153</v>
+      </c>
+      <c r="G272">
+        <v>16106</v>
+      </c>
+      <c r="H272">
+        <v>15891</v>
+      </c>
+      <c r="I272">
+        <v>19437</v>
+      </c>
+      <c r="J272">
+        <v>16881</v>
+      </c>
+      <c r="K272">
+        <v>21474</v>
+      </c>
+      <c r="L272">
+        <v>12769</v>
+      </c>
+      <c r="M272">
+        <v>19228</v>
+      </c>
+      <c r="N272">
+        <v>0</v>
+      </c>
+      <c r="O272">
+        <v>-3</v>
+      </c>
+      <c r="Q272">
+        <v>5</v>
+      </c>
+      <c r="R272">
+        <v>-1</v>
+      </c>
+      <c r="S272">
+        <v>2</v>
+      </c>
+      <c r="U272">
+        <v>0</v>
+      </c>
+      <c r="V272">
+        <v>-3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
take a wild guess.
</commit_message>
<xml_diff>
--- a/datasets/xlsx/CSPreMatchStatistics.xlsx
+++ b/datasets/xlsx/CSPreMatchStatistics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexPost\Repos\HardWareWebsite\datasets\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DF0AF98-610D-4782-A4BD-2D0A3C79626F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF3259FC-EB6E-42DA-99D1-E8C46EAB2D5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -477,7 +477,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V275"/>
+  <dimension ref="A1:V277"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="14.85546875" customWidth="1"/>
@@ -15987,6 +15987,121 @@
         <v>4</v>
       </c>
     </row>
+    <row r="276" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A276">
+        <v>1166</v>
+      </c>
+      <c r="B276">
+        <v>2111</v>
+      </c>
+      <c r="C276">
+        <v>2111</v>
+      </c>
+      <c r="F276">
+        <v>9670</v>
+      </c>
+      <c r="G276">
+        <v>9663</v>
+      </c>
+      <c r="H276">
+        <v>9637</v>
+      </c>
+      <c r="J276">
+        <v>10144</v>
+      </c>
+      <c r="K276">
+        <v>11399</v>
+      </c>
+      <c r="L276">
+        <v>8378</v>
+      </c>
+      <c r="M276">
+        <v>9059</v>
+      </c>
+      <c r="N276">
+        <v>-3</v>
+      </c>
+      <c r="O276">
+        <v>1</v>
+      </c>
+      <c r="Q276">
+        <v>-2</v>
+      </c>
+      <c r="R276">
+        <v>0</v>
+      </c>
+      <c r="S276">
+        <v>-3</v>
+      </c>
+      <c r="U276">
+        <v>-5</v>
+      </c>
+      <c r="V276">
+        <v>-4</v>
+      </c>
+    </row>
+    <row r="277" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A277">
+        <v>1167</v>
+      </c>
+      <c r="B277">
+        <v>2111</v>
+      </c>
+      <c r="C277">
+        <v>5</v>
+      </c>
+      <c r="D277">
+        <v>21729</v>
+      </c>
+      <c r="E277">
+        <v>19594</v>
+      </c>
+      <c r="F277">
+        <v>21418</v>
+      </c>
+      <c r="G277">
+        <v>20768</v>
+      </c>
+      <c r="H277">
+        <v>20109</v>
+      </c>
+      <c r="I277">
+        <v>19200</v>
+      </c>
+      <c r="J277">
+        <v>15510</v>
+      </c>
+      <c r="K277">
+        <v>18132</v>
+      </c>
+      <c r="L277">
+        <v>24225</v>
+      </c>
+      <c r="M277">
+        <v>20454</v>
+      </c>
+      <c r="N277">
+        <v>1</v>
+      </c>
+      <c r="O277">
+        <v>-2</v>
+      </c>
+      <c r="Q277">
+        <v>-3</v>
+      </c>
+      <c r="R277">
+        <v>-5</v>
+      </c>
+      <c r="S277">
+        <v>1</v>
+      </c>
+      <c r="U277">
+        <v>7</v>
+      </c>
+      <c r="V277">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>